<commit_message>
Calculate impact of switching to every 3 days.
</commit_message>
<xml_diff>
--- a/drugs/medicine.xlsx
+++ b/drugs/medicine.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\lucent\health-data\drugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8504D076-10CE-4002-9315-A32EA404B10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B759E786-C734-48BD-B6A0-F852E27A213B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1643" yWindow="862" windowWidth="13117" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1464" yWindow="1464" windowWidth="21504" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="83">
   <si>
     <t>Date</t>
   </si>
@@ -260,6 +260,15 @@
   </si>
   <si>
     <t>389001989216</t>
+  </si>
+  <si>
+    <t>Clicks</t>
+  </si>
+  <si>
+    <t>D965718</t>
+  </si>
+  <si>
+    <t>329426902961</t>
   </si>
 </sst>
 </file>
@@ -271,10 +280,16 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -586,20 +601,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -610,22 +626,25 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>45552.541666666657</v>
       </c>
@@ -635,23 +654,23 @@
       <c r="C2">
         <v>2.5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3">
+      <c r="G2" s="3">
         <v>46102</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>45559.5</v>
       </c>
@@ -661,23 +680,23 @@
       <c r="C3">
         <v>2.5</v>
       </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
       <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="3">
+      <c r="G3" s="3">
         <v>46102</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>45566.5</v>
       </c>
@@ -687,23 +706,23 @@
       <c r="C4">
         <v>2.5</v>
       </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
       <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="3">
+      <c r="G4" s="3">
         <v>46102</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>45573.5</v>
       </c>
@@ -713,23 +732,23 @@
       <c r="C5">
         <v>2.5</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="3">
         <v>46102</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>45580.5</v>
       </c>
@@ -739,23 +758,23 @@
       <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>18</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="3">
         <v>46141</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>45587.5</v>
       </c>
@@ -765,23 +784,23 @@
       <c r="C7">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>22</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="3">
+      <c r="G7" s="3">
         <v>46141</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>45594.583333333343</v>
       </c>
@@ -791,23 +810,23 @@
       <c r="C8">
         <v>5</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>23</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="3">
         <v>46141</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>45601.5</v>
       </c>
@@ -817,23 +836,23 @@
       <c r="C9">
         <v>5</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>24</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="3">
+      <c r="G9" s="3">
         <v>46141</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>45608.5</v>
       </c>
@@ -843,20 +862,20 @@
       <c r="C10">
         <v>5</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>25</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="3">
+      <c r="G10" s="3">
         <v>46139</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>45615.5</v>
       </c>
@@ -866,17 +885,17 @@
       <c r="C11">
         <v>5</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="3">
+      <c r="G11" s="3">
         <v>46139</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>45622.5</v>
       </c>
@@ -886,17 +905,17 @@
       <c r="C12">
         <v>5</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>26</v>
       </c>
-      <c r="F12" s="3">
+      <c r="G12" s="3">
         <v>46139</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>45629.5</v>
       </c>
@@ -906,17 +925,17 @@
       <c r="C13">
         <v>5</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="3">
+      <c r="G13" s="3">
         <v>46139</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>45636.75</v>
       </c>
@@ -926,20 +945,20 @@
       <c r="C14">
         <v>5</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>28</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="3">
+      <c r="G14" s="3">
         <v>46154</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>45645.5</v>
       </c>
@@ -949,23 +968,23 @@
       <c r="C15">
         <v>5</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>31</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>29</v>
       </c>
-      <c r="F15" s="3">
+      <c r="G15" s="3">
         <v>46154</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>45650.583333333343</v>
       </c>
@@ -975,23 +994,23 @@
       <c r="C16">
         <v>5</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>23</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="3">
+      <c r="G16" s="3">
         <v>46154</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>45657.5</v>
       </c>
@@ -1001,23 +1020,23 @@
       <c r="C17">
         <v>5</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>24</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="3">
+      <c r="G17" s="3">
         <v>46154</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>45664.541666666657</v>
       </c>
@@ -1027,23 +1046,23 @@
       <c r="C18">
         <v>5</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>23</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="3">
+      <c r="G18" s="3">
         <v>46154</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>45671.625</v>
       </c>
@@ -1053,23 +1072,23 @@
       <c r="C19">
         <v>5</v>
       </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
       <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="3">
+      <c r="G19" s="3">
         <v>46154</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>45678.645833333343</v>
       </c>
@@ -1079,20 +1098,20 @@
       <c r="C20">
         <v>5</v>
       </c>
-      <c r="D20" t="s">
-        <v>15</v>
-      </c>
       <c r="E20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
         <v>29</v>
       </c>
-      <c r="F20" s="3">
+      <c r="G20" s="3">
         <v>46154</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>45685.541666666657</v>
       </c>
@@ -1102,20 +1121,20 @@
       <c r="C21">
         <v>5</v>
       </c>
-      <c r="D21" t="s">
-        <v>13</v>
-      </c>
       <c r="E21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="3">
+      <c r="G21" s="3">
         <v>46154</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="H21" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>45692.604166666657</v>
       </c>
@@ -1125,20 +1144,20 @@
       <c r="C22">
         <v>5</v>
       </c>
-      <c r="D22" t="s">
-        <v>15</v>
-      </c>
       <c r="E22" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" t="s">
         <v>34</v>
       </c>
-      <c r="F22" s="3">
+      <c r="G22" s="3">
         <v>46178</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>45699.5625</v>
       </c>
@@ -1148,23 +1167,23 @@
       <c r="C23">
         <v>5</v>
       </c>
-      <c r="D23" t="s">
-        <v>13</v>
-      </c>
       <c r="E23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" t="s">
         <v>34</v>
       </c>
-      <c r="F23" s="3">
+      <c r="G23" s="3">
         <v>46178</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>45706.625</v>
       </c>
@@ -1174,23 +1193,23 @@
       <c r="C24">
         <v>5</v>
       </c>
-      <c r="D24" t="s">
-        <v>15</v>
-      </c>
       <c r="E24" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="3">
+      <c r="G24" s="3">
         <v>46178</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>45713.625</v>
       </c>
@@ -1200,23 +1219,23 @@
       <c r="C25">
         <v>5</v>
       </c>
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
       <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" t="s">
         <v>34</v>
       </c>
-      <c r="F25" s="3">
+      <c r="G25" s="3">
         <v>46178</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="H25" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>45720.583333333343</v>
       </c>
@@ -1226,23 +1245,23 @@
       <c r="C26">
         <v>7.5</v>
       </c>
-      <c r="D26" t="s">
-        <v>15</v>
-      </c>
       <c r="E26" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" t="s">
         <v>37</v>
       </c>
-      <c r="F26" s="3">
+      <c r="G26" s="3">
         <v>46258</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="H26" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>45727.645833333343</v>
       </c>
@@ -1252,23 +1271,23 @@
       <c r="C27">
         <v>7.5</v>
       </c>
-      <c r="D27" t="s">
-        <v>13</v>
-      </c>
       <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" t="s">
         <v>37</v>
       </c>
-      <c r="F27" s="3">
+      <c r="G27" s="3">
         <v>46258</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="H27" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>45734.645833333343</v>
       </c>
@@ -1278,23 +1297,23 @@
       <c r="C28">
         <v>7.5</v>
       </c>
-      <c r="D28" t="s">
-        <v>15</v>
-      </c>
       <c r="E28" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" t="s">
         <v>37</v>
       </c>
-      <c r="F28" s="3">
+      <c r="G28" s="3">
         <v>46258</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>45741.583333333343</v>
       </c>
@@ -1304,23 +1323,23 @@
       <c r="C29">
         <v>7.5</v>
       </c>
-      <c r="D29" t="s">
-        <v>13</v>
-      </c>
       <c r="E29" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" t="s">
         <v>37</v>
       </c>
-      <c r="F29" s="3">
+      <c r="G29" s="3">
         <v>46258</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="H29" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>45748.666666666657</v>
       </c>
@@ -1330,23 +1349,23 @@
       <c r="C30">
         <v>7.5</v>
       </c>
-      <c r="D30" t="s">
-        <v>15</v>
-      </c>
       <c r="E30" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" t="s">
         <v>39</v>
       </c>
-      <c r="F30" s="3">
+      <c r="G30" s="3">
         <v>46317</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>45755.8125</v>
       </c>
@@ -1356,23 +1375,23 @@
       <c r="C31">
         <v>7.5</v>
       </c>
-      <c r="D31" t="s">
-        <v>13</v>
-      </c>
       <c r="E31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" t="s">
         <v>39</v>
       </c>
-      <c r="F31" s="3">
+      <c r="G31" s="3">
         <v>46317</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>45762.645833333343</v>
       </c>
@@ -1382,23 +1401,23 @@
       <c r="C32">
         <v>7.5</v>
       </c>
-      <c r="D32" t="s">
-        <v>15</v>
-      </c>
       <c r="E32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" t="s">
         <v>39</v>
       </c>
-      <c r="F32" s="3">
+      <c r="G32" s="3">
         <v>46317</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="H32" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>45769.666666666657</v>
       </c>
@@ -1408,23 +1427,23 @@
       <c r="C33">
         <v>7.5</v>
       </c>
-      <c r="D33" t="s">
-        <v>13</v>
-      </c>
       <c r="E33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" t="s">
         <v>39</v>
       </c>
-      <c r="F33" s="3">
+      <c r="G33" s="3">
         <v>46317</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="H33" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>45776.666666666657</v>
       </c>
@@ -1434,23 +1453,23 @@
       <c r="C34">
         <v>7.5</v>
       </c>
-      <c r="D34" t="s">
-        <v>15</v>
-      </c>
       <c r="E34" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" t="s">
         <v>39</v>
       </c>
-      <c r="F34" s="3">
+      <c r="G34" s="3">
         <v>46317</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="H34" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H34" t="s">
+      <c r="I34" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>45783.708333333343</v>
       </c>
@@ -1460,23 +1479,23 @@
       <c r="C35">
         <v>7.5</v>
       </c>
-      <c r="D35" t="s">
-        <v>13</v>
-      </c>
       <c r="E35" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" t="s">
         <v>39</v>
       </c>
-      <c r="F35" s="3">
+      <c r="G35" s="3">
         <v>46317</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="H35" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>45790.666666666657</v>
       </c>
@@ -1486,20 +1505,20 @@
       <c r="C36">
         <v>7.5</v>
       </c>
-      <c r="D36" t="s">
-        <v>15</v>
-      </c>
       <c r="E36" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" t="s">
         <v>39</v>
       </c>
-      <c r="F36" s="3">
+      <c r="G36" s="3">
         <v>46317</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="H36" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>45797.624999884261</v>
       </c>
@@ -1509,20 +1528,20 @@
       <c r="C37">
         <v>7.5</v>
       </c>
-      <c r="D37" t="s">
-        <v>13</v>
-      </c>
       <c r="E37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" t="s">
         <v>39</v>
       </c>
-      <c r="F37" s="3">
+      <c r="G37" s="3">
         <v>46317</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>45804.666666666657</v>
       </c>
@@ -1532,20 +1551,20 @@
       <c r="C38">
         <v>10</v>
       </c>
-      <c r="D38" t="s">
-        <v>15</v>
-      </c>
       <c r="E38" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" t="s">
         <v>43</v>
       </c>
-      <c r="F38" s="3">
+      <c r="G38" s="3">
         <v>46385</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>45811.625</v>
       </c>
@@ -1555,20 +1574,20 @@
       <c r="C39">
         <v>10</v>
       </c>
-      <c r="D39" t="s">
-        <v>13</v>
-      </c>
       <c r="E39" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" t="s">
         <v>43</v>
       </c>
-      <c r="F39" s="3">
+      <c r="G39" s="3">
         <v>46385</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="H39" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>45818.625</v>
       </c>
@@ -1578,20 +1597,20 @@
       <c r="C40">
         <v>10</v>
       </c>
-      <c r="D40" t="s">
-        <v>15</v>
-      </c>
       <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" t="s">
         <v>43</v>
       </c>
-      <c r="F40" s="3">
+      <c r="G40" s="3">
         <v>46385</v>
       </c>
-      <c r="G40" s="2" t="s">
+      <c r="H40" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>45825.666666666657</v>
       </c>
@@ -1601,20 +1620,20 @@
       <c r="C41">
         <v>10</v>
       </c>
-      <c r="D41" t="s">
-        <v>13</v>
-      </c>
       <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" t="s">
         <v>43</v>
       </c>
-      <c r="F41" s="3">
+      <c r="G41" s="3">
         <v>46385</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="H41" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>45832.70833321759</v>
       </c>
@@ -1624,20 +1643,20 @@
       <c r="C42">
         <v>10</v>
       </c>
-      <c r="D42" t="s">
-        <v>15</v>
-      </c>
       <c r="E42" t="s">
+        <v>15</v>
+      </c>
+      <c r="F42" t="s">
         <v>45</v>
       </c>
-      <c r="F42" s="3">
+      <c r="G42" s="3">
         <v>46317</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="H42" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>45839.666666666657</v>
       </c>
@@ -1647,20 +1666,20 @@
       <c r="C43">
         <v>10</v>
       </c>
-      <c r="D43" t="s">
-        <v>13</v>
-      </c>
       <c r="E43" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" t="s">
         <v>45</v>
       </c>
-      <c r="F43" s="3">
+      <c r="G43" s="3">
         <v>46317</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="H43" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>45846.708333333343</v>
       </c>
@@ -1670,20 +1689,20 @@
       <c r="C44">
         <v>10</v>
       </c>
-      <c r="D44" t="s">
-        <v>15</v>
-      </c>
       <c r="E44" t="s">
+        <v>15</v>
+      </c>
+      <c r="F44" t="s">
         <v>45</v>
       </c>
-      <c r="F44" s="3">
+      <c r="G44" s="3">
         <v>46317</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="H44" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>45853.999305555553</v>
       </c>
@@ -1693,20 +1712,20 @@
       <c r="C45">
         <v>10</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>47</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>45</v>
       </c>
-      <c r="F45" s="3">
+      <c r="G45" s="3">
         <v>46317</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="H45" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>45860.708333333343</v>
       </c>
@@ -1716,20 +1735,20 @@
       <c r="C46">
         <v>10</v>
       </c>
-      <c r="D46" t="s">
-        <v>13</v>
-      </c>
       <c r="E46" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" t="s">
         <v>48</v>
       </c>
-      <c r="F46" s="3">
+      <c r="G46" s="3">
         <v>46457</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="H46" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>45867.8125</v>
       </c>
@@ -1739,20 +1758,20 @@
       <c r="C47">
         <v>10</v>
       </c>
-      <c r="D47" t="s">
-        <v>15</v>
-      </c>
       <c r="E47" t="s">
+        <v>15</v>
+      </c>
+      <c r="F47" t="s">
         <v>48</v>
       </c>
-      <c r="F47" s="3">
+      <c r="G47" s="3">
         <v>46457</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="H47" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>45874.770833333343</v>
       </c>
@@ -1762,20 +1781,20 @@
       <c r="C48">
         <v>10</v>
       </c>
-      <c r="D48" t="s">
-        <v>13</v>
-      </c>
       <c r="E48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" t="s">
         <v>48</v>
       </c>
-      <c r="F48" s="3">
+      <c r="G48" s="3">
         <v>46457</v>
       </c>
-      <c r="G48" s="2" t="s">
+      <c r="H48" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>45881.791666666657</v>
       </c>
@@ -1785,20 +1804,20 @@
       <c r="C49">
         <v>10</v>
       </c>
-      <c r="D49" t="s">
-        <v>15</v>
-      </c>
       <c r="E49" t="s">
+        <v>15</v>
+      </c>
+      <c r="F49" t="s">
         <v>48</v>
       </c>
-      <c r="F49" s="3">
+      <c r="G49" s="3">
         <v>46457</v>
       </c>
-      <c r="G49" s="2" t="s">
+      <c r="H49" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>45888.729166666657</v>
       </c>
@@ -1808,20 +1827,20 @@
       <c r="C50">
         <v>12.5</v>
       </c>
-      <c r="D50" t="s">
-        <v>13</v>
-      </c>
       <c r="E50" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" t="s">
         <v>50</v>
       </c>
-      <c r="F50" s="3">
+      <c r="G50" s="3">
         <v>46513</v>
       </c>
-      <c r="G50" s="2" t="s">
+      <c r="H50" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>45895.75</v>
       </c>
@@ -1831,20 +1850,20 @@
       <c r="C51">
         <v>12.5</v>
       </c>
-      <c r="D51" t="s">
-        <v>15</v>
-      </c>
       <c r="E51" t="s">
+        <v>15</v>
+      </c>
+      <c r="F51" t="s">
         <v>50</v>
       </c>
-      <c r="F51" s="3">
+      <c r="G51" s="3">
         <v>46513</v>
       </c>
-      <c r="G51" s="2" t="s">
+      <c r="H51" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>45902.770833333343</v>
       </c>
@@ -1854,20 +1873,20 @@
       <c r="C52">
         <v>12.5</v>
       </c>
-      <c r="D52" t="s">
-        <v>13</v>
-      </c>
       <c r="E52" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" t="s">
         <v>50</v>
       </c>
-      <c r="F52" s="3">
+      <c r="G52" s="3">
         <v>46513</v>
       </c>
-      <c r="G52" s="2" t="s">
+      <c r="H52" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>45909.791666666657</v>
       </c>
@@ -1877,20 +1896,20 @@
       <c r="C53">
         <v>12.5</v>
       </c>
-      <c r="D53" t="s">
-        <v>15</v>
-      </c>
       <c r="E53" t="s">
+        <v>15</v>
+      </c>
+      <c r="F53" t="s">
         <v>50</v>
       </c>
-      <c r="F53" s="3">
+      <c r="G53" s="3">
         <v>46513</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="H53" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>45916.791666666657</v>
       </c>
@@ -1900,20 +1919,20 @@
       <c r="C54">
         <v>12.5</v>
       </c>
-      <c r="D54" t="s">
-        <v>13</v>
-      </c>
       <c r="E54" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" t="s">
         <v>52</v>
       </c>
-      <c r="F54" s="3">
+      <c r="G54" s="3">
         <v>46516</v>
       </c>
-      <c r="G54" s="2" t="s">
+      <c r="H54" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>45923.791666608799</v>
       </c>
@@ -1923,20 +1942,20 @@
       <c r="C55">
         <v>12.5</v>
       </c>
-      <c r="D55" t="s">
-        <v>15</v>
-      </c>
       <c r="E55" t="s">
+        <v>15</v>
+      </c>
+      <c r="F55" t="s">
         <v>52</v>
       </c>
-      <c r="F55" s="3">
+      <c r="G55" s="3">
         <v>46516</v>
       </c>
-      <c r="G55" s="2" t="s">
+      <c r="H55" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>45930.770833333343</v>
       </c>
@@ -1946,20 +1965,20 @@
       <c r="C56">
         <v>12.5</v>
       </c>
-      <c r="D56" t="s">
-        <v>13</v>
-      </c>
       <c r="E56" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" t="s">
         <v>52</v>
       </c>
-      <c r="F56" s="3">
+      <c r="G56" s="3">
         <v>46516</v>
       </c>
-      <c r="G56" s="2" t="s">
+      <c r="H56" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>45937.791666608799</v>
       </c>
@@ -1969,20 +1988,20 @@
       <c r="C57">
         <v>12.5</v>
       </c>
-      <c r="D57" t="s">
-        <v>15</v>
-      </c>
       <c r="E57" t="s">
+        <v>15</v>
+      </c>
+      <c r="F57" t="s">
         <v>52</v>
       </c>
-      <c r="F57" s="3">
+      <c r="G57" s="3">
         <v>46516</v>
       </c>
-      <c r="G57" s="2" t="s">
+      <c r="H57" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>45944.791666666657</v>
       </c>
@@ -1992,20 +2011,20 @@
       <c r="C58">
         <v>12.5</v>
       </c>
-      <c r="D58" t="s">
-        <v>13</v>
-      </c>
       <c r="E58" t="s">
+        <v>13</v>
+      </c>
+      <c r="F58" t="s">
         <v>50</v>
       </c>
-      <c r="F58" s="3">
+      <c r="G58" s="3">
         <v>46513</v>
       </c>
-      <c r="G58" s="2" t="s">
+      <c r="H58" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>45951.854166666657</v>
       </c>
@@ -2015,20 +2034,20 @@
       <c r="C59">
         <v>12.5</v>
       </c>
-      <c r="D59" t="s">
-        <v>15</v>
-      </c>
       <c r="E59" t="s">
+        <v>15</v>
+      </c>
+      <c r="F59" t="s">
         <v>50</v>
       </c>
-      <c r="F59" s="3">
+      <c r="G59" s="3">
         <v>46513</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="H59" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
         <v>45958.791666666657</v>
       </c>
@@ -2038,20 +2057,20 @@
       <c r="C60">
         <v>12.5</v>
       </c>
-      <c r="D60" t="s">
-        <v>13</v>
-      </c>
       <c r="E60" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" t="s">
         <v>50</v>
       </c>
-      <c r="F60" s="3">
+      <c r="G60" s="3">
         <v>46513</v>
       </c>
-      <c r="G60" s="2" t="s">
+      <c r="H60" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
         <v>45965.75</v>
       </c>
@@ -2061,20 +2080,20 @@
       <c r="C61">
         <v>12.5</v>
       </c>
-      <c r="D61" t="s">
-        <v>15</v>
-      </c>
       <c r="E61" t="s">
+        <v>15</v>
+      </c>
+      <c r="F61" t="s">
         <v>50</v>
       </c>
-      <c r="F61" s="3">
+      <c r="G61" s="3">
         <v>46513</v>
       </c>
-      <c r="G61" s="2" t="s">
+      <c r="H61" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
         <v>45972.708333391201</v>
       </c>
@@ -2084,20 +2103,20 @@
       <c r="C62">
         <v>12.5</v>
       </c>
-      <c r="D62" t="s">
-        <v>13</v>
-      </c>
       <c r="E62" t="s">
+        <v>13</v>
+      </c>
+      <c r="F62" t="s">
         <v>55</v>
       </c>
-      <c r="F62" s="3">
+      <c r="G62" s="3">
         <v>46573</v>
       </c>
-      <c r="G62" s="2" t="s">
+      <c r="H62" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
         <v>45979.75</v>
       </c>
@@ -2107,20 +2126,20 @@
       <c r="C63">
         <v>12.5</v>
       </c>
-      <c r="D63" t="s">
-        <v>15</v>
-      </c>
       <c r="E63" t="s">
+        <v>15</v>
+      </c>
+      <c r="F63" t="s">
         <v>55</v>
       </c>
-      <c r="F63" s="3">
+      <c r="G63" s="3">
         <v>46573</v>
       </c>
-      <c r="G63" s="2" t="s">
+      <c r="H63" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
         <v>45986.8125</v>
       </c>
@@ -2130,20 +2149,20 @@
       <c r="C64">
         <v>12.5</v>
       </c>
-      <c r="D64" t="s">
-        <v>13</v>
-      </c>
       <c r="E64" t="s">
+        <v>13</v>
+      </c>
+      <c r="F64" t="s">
         <v>55</v>
       </c>
-      <c r="F64" s="3">
+      <c r="G64" s="3">
         <v>46573</v>
       </c>
-      <c r="G64" s="2" t="s">
+      <c r="H64" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="1">
         <v>45993.999305555553</v>
       </c>
@@ -2153,20 +2172,20 @@
       <c r="C65">
         <v>12.5</v>
       </c>
-      <c r="D65" t="s">
-        <v>15</v>
-      </c>
       <c r="E65" t="s">
+        <v>15</v>
+      </c>
+      <c r="F65" t="s">
         <v>55</v>
       </c>
-      <c r="F65" s="3">
+      <c r="G65" s="3">
         <v>46573</v>
       </c>
-      <c r="G65" s="2" t="s">
+      <c r="H65" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="1">
         <v>46000.916666666657</v>
       </c>
@@ -2176,20 +2195,20 @@
       <c r="C66">
         <v>12.5</v>
       </c>
-      <c r="D66" t="s">
-        <v>13</v>
-      </c>
       <c r="E66" t="s">
+        <v>13</v>
+      </c>
+      <c r="F66" t="s">
         <v>57</v>
       </c>
-      <c r="F66" s="3">
+      <c r="G66" s="3">
         <v>46530</v>
       </c>
-      <c r="G66" s="2" t="s">
+      <c r="H66" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="1">
         <v>46007.75</v>
       </c>
@@ -2199,20 +2218,20 @@
       <c r="C67">
         <v>12.5</v>
       </c>
-      <c r="D67" t="s">
-        <v>15</v>
-      </c>
       <c r="E67" t="s">
+        <v>15</v>
+      </c>
+      <c r="F67" t="s">
         <v>57</v>
       </c>
-      <c r="F67" s="3">
+      <c r="G67" s="3">
         <v>46530</v>
       </c>
-      <c r="G67" s="2" t="s">
+      <c r="H67" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="1">
         <v>46014.8125</v>
       </c>
@@ -2222,20 +2241,20 @@
       <c r="C68">
         <v>12.5</v>
       </c>
-      <c r="D68" t="s">
-        <v>13</v>
-      </c>
       <c r="E68" t="s">
+        <v>13</v>
+      </c>
+      <c r="F68" t="s">
         <v>57</v>
       </c>
-      <c r="F68" s="3">
+      <c r="G68" s="3">
         <v>46530</v>
       </c>
-      <c r="G68" s="2" t="s">
+      <c r="H68" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="1">
         <v>46021.875</v>
       </c>
@@ -2245,20 +2264,20 @@
       <c r="C69">
         <v>12.5</v>
       </c>
-      <c r="D69" t="s">
-        <v>15</v>
-      </c>
       <c r="E69" t="s">
+        <v>15</v>
+      </c>
+      <c r="F69" t="s">
         <v>57</v>
       </c>
-      <c r="F69" s="3">
+      <c r="G69" s="3">
         <v>46530</v>
       </c>
-      <c r="G69" s="2" t="s">
+      <c r="H69" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="1">
         <v>46028.916666666657</v>
       </c>
@@ -2268,20 +2287,20 @@
       <c r="C70">
         <v>12.5</v>
       </c>
-      <c r="D70" t="s">
-        <v>13</v>
-      </c>
       <c r="E70" t="s">
+        <v>13</v>
+      </c>
+      <c r="F70" t="s">
         <v>59</v>
       </c>
-      <c r="F70" s="3">
+      <c r="G70" s="3">
         <v>46575</v>
       </c>
-      <c r="G70" s="2" t="s">
+      <c r="H70" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="1">
         <v>46035.95833321759</v>
       </c>
@@ -2291,20 +2310,20 @@
       <c r="C71">
         <v>12.5</v>
       </c>
-      <c r="D71" t="s">
-        <v>15</v>
-      </c>
       <c r="E71" t="s">
+        <v>15</v>
+      </c>
+      <c r="F71" t="s">
         <v>59</v>
       </c>
-      <c r="F71" s="3">
+      <c r="G71" s="3">
         <v>46575</v>
       </c>
-      <c r="G71" s="2" t="s">
+      <c r="H71" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="1">
         <v>46042.999305555553</v>
       </c>
@@ -2314,20 +2333,20 @@
       <c r="C72">
         <v>12.5</v>
       </c>
-      <c r="D72" t="s">
-        <v>13</v>
-      </c>
       <c r="E72" t="s">
+        <v>13</v>
+      </c>
+      <c r="F72" t="s">
         <v>59</v>
       </c>
-      <c r="F72" s="3">
+      <c r="G72" s="3">
         <v>46575</v>
       </c>
-      <c r="G72" s="2" t="s">
+      <c r="H72" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="1">
         <v>46049.9375</v>
       </c>
@@ -2337,20 +2356,20 @@
       <c r="C73">
         <v>12.5</v>
       </c>
-      <c r="D73" t="s">
-        <v>15</v>
-      </c>
       <c r="E73" t="s">
+        <v>15</v>
+      </c>
+      <c r="F73" t="s">
         <v>59</v>
       </c>
-      <c r="F73" s="3">
+      <c r="G73" s="3">
         <v>46575</v>
       </c>
-      <c r="G73" s="2" t="s">
+      <c r="H73" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="1">
         <v>46056.9375</v>
       </c>
@@ -2360,20 +2379,20 @@
       <c r="C74">
         <v>12.5</v>
       </c>
-      <c r="D74" t="s">
-        <v>13</v>
-      </c>
       <c r="E74" t="s">
+        <v>13</v>
+      </c>
+      <c r="F74" t="s">
         <v>59</v>
       </c>
-      <c r="F74" s="3">
+      <c r="G74" s="3">
         <v>46575</v>
       </c>
-      <c r="G74" s="2" t="s">
+      <c r="H74" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="1">
         <v>46063.998611111107</v>
       </c>
@@ -2383,20 +2402,20 @@
       <c r="C75">
         <v>12.5</v>
       </c>
-      <c r="D75" t="s">
-        <v>15</v>
-      </c>
       <c r="E75" t="s">
+        <v>15</v>
+      </c>
+      <c r="F75" t="s">
         <v>59</v>
       </c>
-      <c r="F75" s="3">
+      <c r="G75" s="3">
         <v>46575</v>
       </c>
-      <c r="G75" s="2" t="s">
+      <c r="H75" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="1">
         <v>46070.999305555553</v>
       </c>
@@ -2406,20 +2425,20 @@
       <c r="C76">
         <v>12.5</v>
       </c>
-      <c r="D76" t="s">
-        <v>13</v>
-      </c>
       <c r="E76" t="s">
+        <v>13</v>
+      </c>
+      <c r="F76" t="s">
         <v>59</v>
       </c>
-      <c r="F76" s="3">
+      <c r="G76" s="3">
         <v>46575</v>
       </c>
-      <c r="G76" s="2" t="s">
+      <c r="H76" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="1">
         <v>46077.9375</v>
       </c>
@@ -2429,20 +2448,20 @@
       <c r="C77">
         <v>12.5</v>
       </c>
-      <c r="D77" t="s">
-        <v>15</v>
-      </c>
       <c r="E77" t="s">
+        <v>15</v>
+      </c>
+      <c r="F77" t="s">
         <v>59</v>
       </c>
-      <c r="F77" s="3">
+      <c r="G77" s="3">
         <v>46575</v>
       </c>
-      <c r="G77" s="2" t="s">
+      <c r="H77" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="1">
         <v>46084.979166666657</v>
       </c>
@@ -2452,20 +2471,20 @@
       <c r="C78">
         <v>12.5</v>
       </c>
-      <c r="D78" t="s">
-        <v>13</v>
-      </c>
       <c r="E78" t="s">
+        <v>13</v>
+      </c>
+      <c r="F78" t="s">
         <v>77</v>
       </c>
-      <c r="F78" s="3">
+      <c r="G78" s="3">
         <v>46700</v>
       </c>
-      <c r="G78" s="2" t="s">
+      <c r="H78" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="1">
         <v>46091.989583333343</v>
       </c>
@@ -2475,20 +2494,20 @@
       <c r="C79">
         <v>12.5</v>
       </c>
-      <c r="D79" t="s">
-        <v>15</v>
-      </c>
       <c r="E79" t="s">
+        <v>15</v>
+      </c>
+      <c r="F79" t="s">
         <v>77</v>
       </c>
-      <c r="F79" s="3">
+      <c r="G79" s="3">
         <v>46700</v>
       </c>
-      <c r="G79" s="2" t="s">
+      <c r="H79" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="1">
         <v>46098.999305555553</v>
       </c>
@@ -2498,20 +2517,20 @@
       <c r="C80">
         <v>12.5</v>
       </c>
-      <c r="D80" t="s">
-        <v>13</v>
-      </c>
       <c r="E80" t="s">
+        <v>13</v>
+      </c>
+      <c r="F80" t="s">
         <v>77</v>
       </c>
-      <c r="F80" s="3">
+      <c r="G80" s="3">
         <v>46700</v>
       </c>
-      <c r="G80" s="2" t="s">
+      <c r="H80" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="1">
         <v>46105.989583333336</v>
       </c>
@@ -2521,128 +2540,233 @@
       <c r="C81">
         <v>12.5</v>
       </c>
-      <c r="D81" t="s">
-        <v>15</v>
-      </c>
       <c r="E81" t="s">
+        <v>15</v>
+      </c>
+      <c r="F81" t="s">
         <v>77</v>
       </c>
-      <c r="F81" s="3">
+      <c r="G81" s="3">
         <v>46700</v>
       </c>
-      <c r="G81" s="2" t="s">
+      <c r="H81" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A86" s="1">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
+        <v>46113.791666666664</v>
+      </c>
+      <c r="B82" t="s">
+        <v>8</v>
+      </c>
+      <c r="C82">
+        <v>12.5</v>
+      </c>
+      <c r="D82">
+        <v>25</v>
+      </c>
+      <c r="E82" t="s">
+        <v>15</v>
+      </c>
+      <c r="F82" t="s">
+        <v>81</v>
+      </c>
+      <c r="G82" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A83" s="1">
+        <v>46116.677083333336</v>
+      </c>
+      <c r="B83" t="s">
+        <v>8</v>
+      </c>
+      <c r="C83">
+        <v>12.5</v>
+      </c>
+      <c r="D83">
+        <v>25</v>
+      </c>
+      <c r="E83" t="s">
+        <v>13</v>
+      </c>
+      <c r="F83" t="s">
+        <v>81</v>
+      </c>
+      <c r="G83" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A84" s="1">
+        <v>46119.666666666664</v>
+      </c>
+      <c r="B84" t="s">
+        <v>8</v>
+      </c>
+      <c r="C84">
+        <v>12.5</v>
+      </c>
+      <c r="D84">
+        <v>25</v>
+      </c>
+      <c r="E84" t="s">
+        <v>15</v>
+      </c>
+      <c r="F84" t="s">
+        <v>81</v>
+      </c>
+      <c r="G84" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A85" s="1">
+        <v>46122.666666666664</v>
+      </c>
+      <c r="B85" t="s">
+        <v>8</v>
+      </c>
+      <c r="C85">
+        <v>12.5</v>
+      </c>
+      <c r="D85">
+        <v>25</v>
+      </c>
+      <c r="E85" t="s">
+        <v>13</v>
+      </c>
+      <c r="F85" t="s">
+        <v>81</v>
+      </c>
+      <c r="G85" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
         <v>45747.5</v>
-      </c>
-      <c r="B86" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A87" s="1">
-        <v>45748.5</v>
       </c>
       <c r="B87" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="1">
-        <v>45748.875</v>
+        <v>45748.5</v>
       </c>
       <c r="B88" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A90" s="4">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
+        <v>45748.875</v>
+      </c>
+      <c r="B89" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A91" s="4">
         <v>44192.5</v>
-      </c>
-      <c r="B90" t="s">
-        <v>62</v>
-      </c>
-      <c r="D90" t="s">
-        <v>63</v>
-      </c>
-      <c r="E90" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A91" s="4">
-        <v>44214.5</v>
       </c>
       <c r="B91" t="s">
         <v>62</v>
       </c>
-      <c r="D91" t="s">
+      <c r="E91" t="s">
         <v>63</v>
       </c>
-      <c r="E91" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F91" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="4">
-        <v>44463.5</v>
+        <v>44214.5</v>
       </c>
       <c r="B92" t="s">
         <v>62</v>
       </c>
-      <c r="D92" t="s">
+      <c r="E92" t="s">
+        <v>63</v>
+      </c>
+      <c r="F92" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A93" s="4">
+        <v>44463.5</v>
+      </c>
+      <c r="B93" t="s">
+        <v>62</v>
+      </c>
+      <c r="E93" t="s">
         <v>66</v>
       </c>
-      <c r="E92" t="s">
+      <c r="F93" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A93" s="4">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A94" s="4">
         <v>44806.5</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B94" t="s">
         <v>68</v>
       </c>
-      <c r="D93" t="s">
+      <c r="E94" t="s">
         <v>69</v>
       </c>
-      <c r="E93" t="s">
+      <c r="F94" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A94" s="4">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A95" s="4">
         <v>45185.5</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B95" t="s">
         <v>71</v>
       </c>
-      <c r="D94" t="s">
+      <c r="E95" t="s">
         <v>72</v>
       </c>
-      <c r="E94" t="s">
+      <c r="F95" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A95" s="4">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A96" s="4">
         <v>45532.5</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B96" t="s">
         <v>74</v>
       </c>
-      <c r="D95" t="s">
+      <c r="E96" t="s">
         <v>75</v>
       </c>
-      <c r="E95" t="s">
+      <c r="F96" t="s">
         <v>76</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
New Kalman filter splitting FM and LM with a third var to absorb noise.
</commit_message>
<xml_diff>
--- a/drugs/medicine.xlsx
+++ b/drugs/medicine.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\lucent\health-data\drugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B759E786-C734-48BD-B6A0-F852E27A213B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76916C1-98F1-433A-B116-6F55C0749841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1464" yWindow="1464" windowWidth="21504" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2983" yWindow="2983" windowWidth="18514" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="83">
   <si>
     <t>Date</t>
   </si>
@@ -601,21 +601,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I96"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I111"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="18.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.15234375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.69140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.3046875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,7 +644,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>45552.541666666657</v>
       </c>
@@ -670,7 +670,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>45559.5</v>
       </c>
@@ -696,7 +696,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>45566.5</v>
       </c>
@@ -722,7 +722,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>45573.5</v>
       </c>
@@ -748,7 +748,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>45580.5</v>
       </c>
@@ -774,7 +774,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>45587.5</v>
       </c>
@@ -800,7 +800,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>45594.583333333343</v>
       </c>
@@ -826,7 +826,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>45601.5</v>
       </c>
@@ -852,7 +852,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>45608.5</v>
       </c>
@@ -875,7 +875,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>45615.5</v>
       </c>
@@ -895,7 +895,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>45622.5</v>
       </c>
@@ -915,7 +915,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>45629.5</v>
       </c>
@@ -935,7 +935,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>45636.75</v>
       </c>
@@ -958,7 +958,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>45645.5</v>
       </c>
@@ -984,7 +984,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>45650.583333333343</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>45657.5</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>45664.541666666657</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>45671.625</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>45678.645833333343</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>45685.541666666657</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A22" s="1">
         <v>45692.604166666657</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A23" s="1">
         <v>45699.5625</v>
       </c>
@@ -1183,7 +1183,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A24" s="1">
         <v>45706.625</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A25" s="1">
         <v>45713.625</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A26" s="1">
         <v>45720.583333333343</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A27" s="1">
         <v>45727.645833333343</v>
       </c>
@@ -1287,7 +1287,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A28" s="1">
         <v>45734.645833333343</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A29" s="1">
         <v>45741.583333333343</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A30" s="1">
         <v>45748.666666666657</v>
       </c>
@@ -1365,7 +1365,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A31" s="1">
         <v>45755.8125</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A32" s="1">
         <v>45762.645833333343</v>
       </c>
@@ -1417,7 +1417,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A33" s="1">
         <v>45769.666666666657</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A34" s="1">
         <v>45776.666666666657</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A35" s="1">
         <v>45783.708333333343</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A36" s="1">
         <v>45790.666666666657</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A37" s="1">
         <v>45797.624999884261</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A38" s="1">
         <v>45804.666666666657</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A39" s="1">
         <v>45811.625</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A40" s="1">
         <v>45818.625</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A41" s="1">
         <v>45825.666666666657</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A42" s="1">
         <v>45832.70833321759</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A43" s="1">
         <v>45839.666666666657</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A44" s="1">
         <v>45846.708333333343</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A45" s="1">
         <v>45853.999305555553</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A46" s="1">
         <v>45860.708333333343</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A47" s="1">
         <v>45867.8125</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A48" s="1">
         <v>45874.770833333343</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A49" s="1">
         <v>45881.791666666657</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A50" s="1">
         <v>45888.729166666657</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A51" s="1">
         <v>45895.75</v>
       </c>
@@ -1863,7 +1863,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A52" s="1">
         <v>45902.770833333343</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A53" s="1">
         <v>45909.791666666657</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A54" s="1">
         <v>45916.791666666657</v>
       </c>
@@ -1932,7 +1932,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A55" s="1">
         <v>45923.791666608799</v>
       </c>
@@ -1955,7 +1955,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A56" s="1">
         <v>45930.770833333343</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A57" s="1">
         <v>45937.791666608799</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A58" s="1">
         <v>45944.791666666657</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A59" s="1">
         <v>45951.854166666657</v>
       </c>
@@ -2047,7 +2047,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A60" s="1">
         <v>45958.791666666657</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A61" s="1">
         <v>45965.75</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A62" s="1">
         <v>45972.708333391201</v>
       </c>
@@ -2116,7 +2116,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A63" s="1">
         <v>45979.75</v>
       </c>
@@ -2139,7 +2139,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A64" s="1">
         <v>45986.8125</v>
       </c>
@@ -2162,7 +2162,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A65" s="1">
         <v>45993.999305555553</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A66" s="1">
         <v>46000.916666666657</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A67" s="1">
         <v>46007.75</v>
       </c>
@@ -2231,7 +2231,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A68" s="1">
         <v>46014.8125</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A69" s="1">
         <v>46021.875</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A70" s="1">
         <v>46028.916666666657</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A71" s="1">
         <v>46035.95833321759</v>
       </c>
@@ -2323,7 +2323,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A72" s="1">
         <v>46042.999305555553</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A73" s="1">
         <v>46049.9375</v>
       </c>
@@ -2369,7 +2369,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A74" s="1">
         <v>46056.9375</v>
       </c>
@@ -2392,7 +2392,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A75" s="1">
         <v>46063.998611111107</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A76" s="1">
         <v>46070.999305555553</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A77" s="1">
         <v>46077.9375</v>
       </c>
@@ -2461,7 +2461,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A78" s="1">
         <v>46084.979166666657</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A79" s="1">
         <v>46091.989583333343</v>
       </c>
@@ -2507,7 +2507,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A80" s="1">
         <v>46098.999305555553</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A81" s="1">
         <v>46105.989583333336</v>
       </c>
@@ -2553,7 +2553,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A82" s="1">
         <v>46113.791666666664</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A83" s="1">
         <v>46116.677083333336</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A84" s="1">
         <v>46119.666666666664</v>
       </c>
@@ -2631,7 +2631,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A85" s="1">
         <v>46122.666666666664</v>
       </c>
@@ -2657,111 +2657,527 @@
         <v>82</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A86" s="1">
+        <v>46125.8125</v>
+      </c>
+      <c r="B86" t="s">
+        <v>8</v>
+      </c>
+      <c r="C86">
+        <v>12.5</v>
+      </c>
+      <c r="D86">
+        <v>25</v>
+      </c>
+      <c r="E86" t="s">
+        <v>15</v>
+      </c>
+      <c r="F86" t="s">
+        <v>81</v>
+      </c>
+      <c r="G86" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A87" s="1">
+        <v>46128.666666608799</v>
+      </c>
+      <c r="B87" t="s">
+        <v>8</v>
+      </c>
+      <c r="C87">
+        <v>12.5</v>
+      </c>
+      <c r="D87">
+        <v>25</v>
+      </c>
+      <c r="E87" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87" t="s">
+        <v>81</v>
+      </c>
+      <c r="G87" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H87" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A88" s="1">
+        <v>46131.666666608799</v>
+      </c>
+      <c r="B88" t="s">
+        <v>8</v>
+      </c>
+      <c r="C88">
+        <v>12.5</v>
+      </c>
+      <c r="D88">
+        <v>25</v>
+      </c>
+      <c r="E88" t="s">
+        <v>15</v>
+      </c>
+      <c r="F88" t="s">
+        <v>81</v>
+      </c>
+      <c r="G88" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A89" s="1">
+        <v>46134.6875</v>
+      </c>
+      <c r="B89" t="s">
+        <v>8</v>
+      </c>
+      <c r="C89">
+        <v>12.5</v>
+      </c>
+      <c r="D89">
+        <v>25</v>
+      </c>
+      <c r="E89" t="s">
+        <v>13</v>
+      </c>
+      <c r="F89" t="s">
+        <v>81</v>
+      </c>
+      <c r="G89" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H89" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A90" s="1">
+        <v>46137.708333333336</v>
+      </c>
+      <c r="B90" t="s">
+        <v>8</v>
+      </c>
+      <c r="C90">
+        <v>12.5</v>
+      </c>
+      <c r="D90">
+        <v>25</v>
+      </c>
+      <c r="E90" t="s">
+        <v>15</v>
+      </c>
+      <c r="F90" t="s">
+        <v>81</v>
+      </c>
+      <c r="G90" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A91" s="1">
+        <v>46140.666666608799</v>
+      </c>
+      <c r="B91" t="s">
+        <v>8</v>
+      </c>
+      <c r="C91">
+        <v>12.5</v>
+      </c>
+      <c r="D91">
+        <v>25</v>
+      </c>
+      <c r="E91" t="s">
+        <v>13</v>
+      </c>
+      <c r="F91" t="s">
+        <v>81</v>
+      </c>
+      <c r="G91" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H91" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A92" s="1">
+        <v>46143.666666608799</v>
+      </c>
+      <c r="B92" t="s">
+        <v>8</v>
+      </c>
+      <c r="C92">
+        <v>12.5</v>
+      </c>
+      <c r="D92">
+        <v>25</v>
+      </c>
+      <c r="E92" t="s">
+        <v>15</v>
+      </c>
+      <c r="F92" t="s">
+        <v>81</v>
+      </c>
+      <c r="G92" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A93" s="1">
+        <v>46146.666666608799</v>
+      </c>
+      <c r="B93" t="s">
+        <v>8</v>
+      </c>
+      <c r="C93">
+        <v>12.5</v>
+      </c>
+      <c r="D93">
+        <v>25</v>
+      </c>
+      <c r="E93" t="s">
+        <v>13</v>
+      </c>
+      <c r="F93" t="s">
+        <v>81</v>
+      </c>
+      <c r="G93" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H93" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A94" s="1">
+        <v>46149.666666608799</v>
+      </c>
+      <c r="B94" t="s">
+        <v>8</v>
+      </c>
+      <c r="C94">
+        <v>12.5</v>
+      </c>
+      <c r="D94">
+        <v>25</v>
+      </c>
+      <c r="E94" t="s">
+        <v>15</v>
+      </c>
+      <c r="F94" t="s">
+        <v>81</v>
+      </c>
+      <c r="G94" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A95" s="1">
+        <v>46152.666666608799</v>
+      </c>
+      <c r="B95" t="s">
+        <v>8</v>
+      </c>
+      <c r="C95">
+        <v>12.5</v>
+      </c>
+      <c r="D95">
+        <v>25</v>
+      </c>
+      <c r="E95" t="s">
+        <v>13</v>
+      </c>
+      <c r="F95" t="s">
+        <v>81</v>
+      </c>
+      <c r="G95" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H95" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A96" s="1">
+        <v>46155.666666608799</v>
+      </c>
+      <c r="B96" t="s">
+        <v>8</v>
+      </c>
+      <c r="C96">
+        <v>12.5</v>
+      </c>
+      <c r="D96">
+        <v>25</v>
+      </c>
+      <c r="E96" t="s">
+        <v>15</v>
+      </c>
+      <c r="F96" t="s">
+        <v>81</v>
+      </c>
+      <c r="G96" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H96" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A97" s="1">
+        <v>46158.666666608799</v>
+      </c>
+      <c r="B97" t="s">
+        <v>8</v>
+      </c>
+      <c r="C97">
+        <v>12.5</v>
+      </c>
+      <c r="D97">
+        <v>25</v>
+      </c>
+      <c r="E97" t="s">
+        <v>13</v>
+      </c>
+      <c r="F97" t="s">
+        <v>81</v>
+      </c>
+      <c r="G97" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H97" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A98" s="1">
+        <v>46161.666666608799</v>
+      </c>
+      <c r="B98" t="s">
+        <v>8</v>
+      </c>
+      <c r="C98">
+        <v>12.5</v>
+      </c>
+      <c r="D98">
+        <v>25</v>
+      </c>
+      <c r="E98" t="s">
+        <v>15</v>
+      </c>
+      <c r="F98" t="s">
+        <v>81</v>
+      </c>
+      <c r="G98" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A99" s="1">
+        <v>46164.666666666664</v>
+      </c>
+      <c r="B99" t="s">
+        <v>8</v>
+      </c>
+      <c r="C99">
+        <v>12.5</v>
+      </c>
+      <c r="D99">
+        <v>25</v>
+      </c>
+      <c r="E99" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" t="s">
+        <v>81</v>
+      </c>
+      <c r="G99" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H99" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A100" s="1">
+        <v>46167.666666666664</v>
+      </c>
+      <c r="B100" t="s">
+        <v>8</v>
+      </c>
+      <c r="C100">
+        <v>12.5</v>
+      </c>
+      <c r="D100">
+        <v>25</v>
+      </c>
+      <c r="E100" t="s">
+        <v>15</v>
+      </c>
+      <c r="F100" t="s">
+        <v>81</v>
+      </c>
+      <c r="G100" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A101" s="1">
+        <v>46170.666666608799</v>
+      </c>
+      <c r="B101" t="s">
+        <v>8</v>
+      </c>
+      <c r="C101">
+        <v>12.5</v>
+      </c>
+      <c r="D101">
+        <v>25</v>
+      </c>
+      <c r="E101" t="s">
+        <v>13</v>
+      </c>
+      <c r="F101" t="s">
+        <v>81</v>
+      </c>
+      <c r="G101" s="3">
+        <v>46567</v>
+      </c>
+      <c r="H101" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A102" s="1">
         <v>45747.5</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B102" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A88" s="1">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A103" s="1">
         <v>45748.5</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B103" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A89" s="1">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A104" s="1">
         <v>45748.875</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B104" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A91" s="4">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A106" s="4">
         <v>44192.5</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B106" t="s">
         <v>62</v>
       </c>
-      <c r="E91" t="s">
+      <c r="E106" t="s">
         <v>63</v>
       </c>
-      <c r="F91" t="s">
+      <c r="F106" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A92" s="4">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A107" s="4">
         <v>44214.5</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B107" t="s">
         <v>62</v>
       </c>
-      <c r="E92" t="s">
+      <c r="E107" t="s">
         <v>63</v>
       </c>
-      <c r="F92" t="s">
+      <c r="F107" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A93" s="4">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A108" s="4">
         <v>44463.5</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B108" t="s">
         <v>62</v>
       </c>
-      <c r="E93" t="s">
+      <c r="E108" t="s">
         <v>66</v>
       </c>
-      <c r="F93" t="s">
+      <c r="F108" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A94" s="4">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A109" s="4">
         <v>44806.5</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B109" t="s">
         <v>68</v>
       </c>
-      <c r="E94" t="s">
+      <c r="E109" t="s">
         <v>69</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F109" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A95" s="4">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A110" s="4">
         <v>45185.5</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B110" t="s">
         <v>71</v>
       </c>
-      <c r="E95" t="s">
+      <c r="E110" t="s">
         <v>72</v>
       </c>
-      <c r="F95" t="s">
+      <c r="F110" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A96" s="4">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A111" s="4">
         <v>45532.5</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B111" t="s">
         <v>74</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E111" t="s">
         <v>75</v>
       </c>
-      <c r="F96" t="s">
+      <c r="F111" t="s">
         <v>76</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise set point framework with intake calibration and new behavioral tests.
</commit_message>
<xml_diff>
--- a/drugs/medicine.xlsx
+++ b/drugs/medicine.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\lucent\health-data\drugs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76916C1-98F1-433A-B116-6F55C0749841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F2D82F-92C6-40CB-BA5F-D9E04EEC2A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2983" yWindow="2983" windowWidth="18514" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1886" yWindow="720" windowWidth="21737" windowHeight="14709" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="87">
   <si>
     <t>Date</t>
   </si>
@@ -269,6 +269,18 @@
   </si>
   <si>
     <t>329426902961</t>
+  </si>
+  <si>
+    <t>302201452706</t>
+  </si>
+  <si>
+    <t>D969425D</t>
+  </si>
+  <si>
+    <t>D969425E</t>
+  </si>
+  <si>
+    <t>356263347017</t>
   </si>
 </sst>
 </file>
@@ -601,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I111"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.15234375" style="1" bestFit="1" customWidth="1"/>
@@ -2789,7 +2801,7 @@
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A91" s="1">
-        <v>46140.666666608799</v>
+        <v>46140.729166666664</v>
       </c>
       <c r="B91" t="s">
         <v>8</v>
@@ -2815,13 +2827,13 @@
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A92" s="1">
-        <v>46143.666666608799</v>
+        <v>46143.708333333336</v>
       </c>
       <c r="B92" t="s">
         <v>8</v>
       </c>
       <c r="C92">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D92">
         <v>25</v>
@@ -2830,24 +2842,24 @@
         <v>15</v>
       </c>
       <c r="F92" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G92" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A93" s="1">
-        <v>46146.666666608799</v>
+        <v>46146.708333333336</v>
       </c>
       <c r="B93" t="s">
         <v>8</v>
       </c>
       <c r="C93">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D93">
         <v>25</v>
@@ -2856,24 +2868,24 @@
         <v>13</v>
       </c>
       <c r="F93" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G93" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A94" s="1">
-        <v>46149.666666608799</v>
+        <v>46149.6875</v>
       </c>
       <c r="B94" t="s">
         <v>8</v>
       </c>
       <c r="C94">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D94">
         <v>25</v>
@@ -2882,24 +2894,24 @@
         <v>15</v>
       </c>
       <c r="F94" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G94" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A95" s="1">
-        <v>46152.666666608799</v>
+        <v>46152.729166666664</v>
       </c>
       <c r="B95" t="s">
         <v>8</v>
       </c>
       <c r="C95">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D95">
         <v>25</v>
@@ -2908,24 +2920,24 @@
         <v>13</v>
       </c>
       <c r="F95" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G95" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A96" s="1">
-        <v>46155.666666608799</v>
+        <v>46155.708333333336</v>
       </c>
       <c r="B96" t="s">
         <v>8</v>
       </c>
       <c r="C96">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D96">
         <v>25</v>
@@ -2934,24 +2946,24 @@
         <v>15</v>
       </c>
       <c r="F96" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G96" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A97" s="1">
-        <v>46158.666666608799</v>
+        <v>46158.729166666664</v>
       </c>
       <c r="B97" t="s">
         <v>8</v>
       </c>
       <c r="C97">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D97">
         <v>25</v>
@@ -2960,24 +2972,24 @@
         <v>13</v>
       </c>
       <c r="F97" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G97" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A98" s="1">
-        <v>46161.666666608799</v>
+        <v>46161.729166666664</v>
       </c>
       <c r="B98" t="s">
         <v>8</v>
       </c>
       <c r="C98">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D98">
         <v>25</v>
@@ -2986,24 +2998,24 @@
         <v>15</v>
       </c>
       <c r="F98" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G98" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A99" s="1">
-        <v>46164.666666666664</v>
+        <v>46164.854166666664</v>
       </c>
       <c r="B99" t="s">
         <v>8</v>
       </c>
       <c r="C99">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D99">
         <v>25</v>
@@ -3012,24 +3024,24 @@
         <v>13</v>
       </c>
       <c r="F99" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G99" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H99" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A100" s="1">
-        <v>46167.666666666664</v>
+        <v>46167.791666666664</v>
       </c>
       <c r="B100" t="s">
         <v>8</v>
       </c>
       <c r="C100">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D100">
         <v>25</v>
@@ -3038,24 +3050,24 @@
         <v>15</v>
       </c>
       <c r="F100" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G100" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H100" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A101" s="1">
-        <v>46170.666666608799</v>
+        <v>46171.833333333336</v>
       </c>
       <c r="B101" t="s">
         <v>8</v>
       </c>
       <c r="C101">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="D101">
         <v>25</v>
@@ -3064,120 +3076,380 @@
         <v>13</v>
       </c>
       <c r="F101" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G101" s="3">
-        <v>46567</v>
+        <v>46710</v>
       </c>
       <c r="H101" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A102" s="1">
-        <v>45747.5</v>
+        <v>46175.8125</v>
       </c>
       <c r="B102" t="s">
-        <v>61</v>
+        <v>8</v>
+      </c>
+      <c r="C102">
+        <v>15</v>
+      </c>
+      <c r="D102">
+        <v>25</v>
+      </c>
+      <c r="E102" t="s">
+        <v>15</v>
+      </c>
+      <c r="F102" t="s">
+        <v>85</v>
+      </c>
+      <c r="G102" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A103" s="1">
-        <v>45748.5</v>
+        <v>46179.854166666664</v>
       </c>
       <c r="B103" t="s">
-        <v>61</v>
+        <v>8</v>
+      </c>
+      <c r="C103">
+        <v>15</v>
+      </c>
+      <c r="D103">
+        <v>25</v>
+      </c>
+      <c r="E103" t="s">
+        <v>13</v>
+      </c>
+      <c r="F103" t="s">
+        <v>85</v>
+      </c>
+      <c r="G103" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H103" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A104" s="1">
+        <v>46183.854166666664</v>
+      </c>
+      <c r="B104" t="s">
+        <v>8</v>
+      </c>
+      <c r="C104">
+        <v>15</v>
+      </c>
+      <c r="D104">
+        <v>25</v>
+      </c>
+      <c r="E104" t="s">
+        <v>15</v>
+      </c>
+      <c r="F104" t="s">
+        <v>85</v>
+      </c>
+      <c r="G104" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H104" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A105" s="1">
+        <v>46187.833333333336</v>
+      </c>
+      <c r="B105" t="s">
+        <v>8</v>
+      </c>
+      <c r="C105">
+        <v>15</v>
+      </c>
+      <c r="D105">
+        <v>25</v>
+      </c>
+      <c r="E105" t="s">
+        <v>13</v>
+      </c>
+      <c r="F105" t="s">
+        <v>85</v>
+      </c>
+      <c r="G105" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H105" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A106" s="1">
+        <v>46191.854166666664</v>
+      </c>
+      <c r="B106" t="s">
+        <v>8</v>
+      </c>
+      <c r="C106">
+        <v>15</v>
+      </c>
+      <c r="D106">
+        <v>25</v>
+      </c>
+      <c r="E106" t="s">
+        <v>15</v>
+      </c>
+      <c r="F106" t="s">
+        <v>85</v>
+      </c>
+      <c r="G106" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H106" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A107" s="1">
+        <v>46195.895833333336</v>
+      </c>
+      <c r="B107" t="s">
+        <v>8</v>
+      </c>
+      <c r="C107">
+        <v>15</v>
+      </c>
+      <c r="D107">
+        <v>25</v>
+      </c>
+      <c r="E107" t="s">
+        <v>13</v>
+      </c>
+      <c r="F107" t="s">
+        <v>85</v>
+      </c>
+      <c r="G107" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H107" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A108" s="1">
+        <v>46199.8125</v>
+      </c>
+      <c r="B108" t="s">
+        <v>8</v>
+      </c>
+      <c r="C108">
+        <v>15</v>
+      </c>
+      <c r="D108">
+        <v>25</v>
+      </c>
+      <c r="E108" t="s">
+        <v>15</v>
+      </c>
+      <c r="F108" t="s">
+        <v>85</v>
+      </c>
+      <c r="G108" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H108" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A109" s="1">
+        <v>46203.999305555553</v>
+      </c>
+      <c r="B109" t="s">
+        <v>8</v>
+      </c>
+      <c r="C109">
+        <v>15</v>
+      </c>
+      <c r="D109">
+        <v>25</v>
+      </c>
+      <c r="E109" t="s">
+        <v>13</v>
+      </c>
+      <c r="F109" t="s">
+        <v>85</v>
+      </c>
+      <c r="G109" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H109" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A110" s="1">
+        <v>46207.9375</v>
+      </c>
+      <c r="B110" t="s">
+        <v>8</v>
+      </c>
+      <c r="C110">
+        <v>15</v>
+      </c>
+      <c r="D110">
+        <v>25</v>
+      </c>
+      <c r="E110" t="s">
+        <v>15</v>
+      </c>
+      <c r="F110" t="s">
+        <v>85</v>
+      </c>
+      <c r="G110" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H110" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A111" s="1">
+        <v>46211.875</v>
+      </c>
+      <c r="B111" t="s">
+        <v>8</v>
+      </c>
+      <c r="C111">
+        <v>15</v>
+      </c>
+      <c r="D111">
+        <v>25</v>
+      </c>
+      <c r="E111" t="s">
+        <v>13</v>
+      </c>
+      <c r="F111" t="s">
+        <v>85</v>
+      </c>
+      <c r="G111" s="3">
+        <v>46710</v>
+      </c>
+      <c r="H111" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A112" s="1">
+        <v>45747.5</v>
+      </c>
+      <c r="B112" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A113" s="1">
+        <v>45748.5</v>
+      </c>
+      <c r="B113" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A114" s="1">
         <v>45748.875</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B114" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A106" s="4">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A116" s="4">
         <v>44192.5</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B116" t="s">
         <v>62</v>
       </c>
-      <c r="E106" t="s">
+      <c r="E116" t="s">
         <v>63</v>
       </c>
-      <c r="F106" t="s">
+      <c r="F116" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A107" s="4">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A117" s="4">
         <v>44214.5</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B117" t="s">
         <v>62</v>
       </c>
-      <c r="E107" t="s">
+      <c r="E117" t="s">
         <v>63</v>
       </c>
-      <c r="F107" t="s">
+      <c r="F117" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A108" s="4">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A118" s="4">
         <v>44463.5</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B118" t="s">
         <v>62</v>
       </c>
-      <c r="E108" t="s">
+      <c r="E118" t="s">
         <v>66</v>
       </c>
-      <c r="F108" t="s">
+      <c r="F118" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A109" s="4">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A119" s="4">
         <v>44806.5</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B119" t="s">
         <v>68</v>
       </c>
-      <c r="E109" t="s">
+      <c r="E119" t="s">
         <v>69</v>
       </c>
-      <c r="F109" t="s">
+      <c r="F119" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A110" s="4">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A120" s="4">
         <v>45185.5</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B120" t="s">
         <v>71</v>
       </c>
-      <c r="E110" t="s">
+      <c r="E120" t="s">
         <v>72</v>
       </c>
-      <c r="F110" t="s">
+      <c r="F120" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A111" s="4">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A121" s="4">
         <v>45532.5</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B121" t="s">
         <v>74</v>
       </c>
-      <c r="E111" t="s">
+      <c r="E121" t="s">
         <v>75</v>
       </c>
-      <c r="F111" t="s">
+      <c r="F121" t="s">
         <v>76</v>
       </c>
     </row>

</xml_diff>